<commit_message>
Add pixel-regression test harness (Step 0 of multi-type refactor)
tests/cases.py builds six synthetic scenarios (EN/ES, filtered/unfiltered,
missing parameter, all-pass/all-fail, both disinfectants) and drives the
real pipeline end to end. tests/compare_pdf.py is the pass/fail gate
(page count, paper size, exact pixel bytes); tests/compare_dom.py is a
diagnostic structural diff. tests/baseline/ holds the current output,
captured from synthetic data only, as the reference every later refactor
step must reproduce exactly.

Verified: --capture-baseline and --verify both run clean, and a repeat
--verify run confirms the pipeline is deterministic (zero pixel diff on
an unchanged rerun).
</commit_message>
<xml_diff>
--- a/data/reference/translations.xlsx
+++ b/data/reference/translations.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B264"/>
+  <dimension ref="A1:B277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,3158 +443,3314 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>(512) 272-5555</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>(512) 272-5555</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/26/2025</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>09/07/2024</t>
+          <t>01/15/2025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09/07/2024</t>
+          <t>15/01/2025</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>07/26/2025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>26/07/2025</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1. Test Results Overview</t>
+          <t>09/07/2024</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1. Resumen de los resultados de la prueba</t>
+          <t>09/07/2024</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10/07/2024</t>
+          <t>1. Test Results Overview</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10/07/2024</t>
+          <t>1. Resumen de los resultados de la prueba</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>11/01/2024</t>
+          <t>10/07/2024</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11/01/2024</t>
+          <t>10/07/2024</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>100 W. Center Street | Kyle, TX 78640</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05/11/2025</t>
+          <t>100 W. Center Street | Kyle, Texas 78640</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11/01/2024</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11/01/2024</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>05/11/2025</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2. Detailed Test Results</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2. Resultados detallados de la prueba</t>
+          <t>16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2024-09-07 00:00:00</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-09-07 00:00:00</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2024-10-07 00:00:00</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-10-07 00:00:00</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2024-11-01 00:00:00</t>
+          <t>2. Detailed Test Results</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-11-01 00:00:00</t>
+          <t>2. Resultados detallados de la prueba</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2024-09-07 00:00:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2024-09-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3. Concerns and questions</t>
+          <t>2024-10-07 00:00:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3. Preocupaciones y preguntas</t>
+          <t>2024-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2024-11-01 00:00:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2024-11-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4. Learn About Your Report</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>4. Más información sobre su informe</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>415 Old Austin Hwy Drawer P, Bastrop, TX 78602</t>
+          <t>3. Concerns and questions</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>415 Old Austin Hwy Cajón P, Bastrop, TX 78602</t>
+          <t>3. Preocupaciones y preguntas</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>512-284-3168</t>
+          <t>4. Learn About Your Report</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>512-284-3168</t>
+          <t>4. Más información sobre su informe</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>512-304-0354</t>
+          <t>415 Old Austin Hwy Drawer P, Bastrop, TX 78602</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>512-304-0354</t>
+          <t>415 Old Austin Hwy Cajón P, Bastrop, TX 78602</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>512-339-2929</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>512-339-2929</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>512-398-4748</t>
+          <t>512-262-3024</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>512-398-4748</t>
+          <t>512-262-3024</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>512-972-0012</t>
+          <t>512-284-3168</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>512-972-0012</t>
+          <t>512-284-3168</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>512-304-0354</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>512-304-0354</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6 out of 7 parameters are within acceptable range.</t>
+          <t>512-339-2929</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>6 de 7 parámetros están dentro del rango aceptable.</t>
+          <t>512-339-2929</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>625 E. 10th St. Austin, TX 78701</t>
+          <t>512-398-4748</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>625 E. 10th St. Austin, TX 78701</t>
+          <t>512-398-4748</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>512-972-0012</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>512-972-0012</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7 out of 7 parameters are within acceptable range.</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7 de 7 parámetros están dentro del rango aceptable.</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6 out of 7 parameters are within acceptable range.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6 de 7 parámetros están dentro del rango aceptable.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8 out of 8 parameters are within acceptable range.</t>
+          <t>625 E. 10th St. Austin, TX 78701</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>8 de 8 parámetros están dentro del rango aceptable.</t>
+          <t>625 E. 10th St. Austin, TX 78701</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8870 Camino Real Uhland, Texas 78640</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>8870 Camino Real Uhland, Texas 78640</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7 out of 7 parameters are within acceptable range.</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7 de 7 parámetros están dentro del rango aceptable.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>A certain amount of disinfectant is needed when the water enters your home. This helps make sure no harmful bacteria grows between the treatment plant and your home.</t>
+          <t>7 out of 8 parameters are within acceptable range.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Se necesita una cierta cantidad de desinfectante cuando el agua entra en su hogar. Esto ayuda a asegurar que no crezcan bacterias dañinas entre la planta de tratamiento y su hogar.</t>
+          <t>7 de 8 parámetros están dentro del rango aceptable.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Acceptable Range</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Rango normal</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Acceptable range</t>
+          <t>8 out of 8 parameters are within acceptable range.</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Rango normal</t>
+          <t>8 de 8 parámetros están dentro del rango aceptable.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Aligns with the WCWH average measurements in your area</t>
+          <t>8870 Camino Real Uhland, Texas 78640</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Se alinea con las medidas promedio de NCNS en su área</t>
+          <t>8870 Camino Real Uhland, Texas 78640</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Amoníaco</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Anonymous report available</t>
+          <t>A certain amount of disinfectant is needed when the water enters your home. This helps make sure no harmful bacteria grows between the treatment plant and your home.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Informe anónimo disponible</t>
+          <t>Se necesita una cierta cantidad de desinfectante cuando el agua entra en su hogar. Esto ayuda a asegurar que no crezcan bacterias dañinas entre la planta de tratamiento y su hogar.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Aqua WSC</t>
+          <t>Acceptable Range</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Aqua WSC</t>
+          <t>Rango normal</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>As a participant in the WCWH study, our doors are always open for you. Don't hesitate to contact us with any questions or concerns about your water quality report.</t>
+          <t>Acceptable range</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Como participante en el estudio NCNS, nuestras puertas siempre están abiertas para usted. No dude en ponerse en contacto con nosotros si tiene alguna pregunta o inquietud acerca de su informe de calidad del agua.</t>
+          <t>Rango normal</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>As of February 2025, we have collected:</t>
+          <t>Aligns with the WCWH average measurements in your area</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>En febrero de 2025, hemos recopilado:</t>
+          <t>Se alinea con las medidas promedio de NCNS en su área</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>As of June 2024, we have collected:</t>
+          <t>Ammonia</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>En junio de 2024, hemos recopilado:</t>
+          <t>Amoníaco</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Austin Water</t>
+          <t>Anonymous report available</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Austin water</t>
+          <t>Informe anónimo disponible</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Average community level</t>
+          <t>Aqua WSC</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad</t>
+          <t>Aqua WSC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Average community level (NTU)</t>
+          <t>As a participant in the WCWH study, our doors are always open for you. Don't hesitate to contact us with any questions or concerns about your water quality report.</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad (NTU)</t>
+          <t>Como participante en el estudio NCNS, nuestras puertas siempre están abiertas para usted. No dude en ponerse en contacto con nosotros si tiene alguna pregunta o inquietud acerca de su informe de calidad del agua.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Average community level (mg/L)</t>
+          <t>As of February 2025, we have collected:</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad (mg/L)</t>
+          <t>En febrero de 2025, hemos recopilado:</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Average community level for kitchen tap</t>
+          <t>As of June 2024, we have collected:</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad para el grifo de cocina</t>
+          <t>En junio de 2024, hemos recopilado:</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Average community level for kitchen tap (NTU)</t>
+          <t>Austin Water</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad para cocina de cocina (NTU)</t>
+          <t>Austin water</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Average community level for kitchen tap (mg/L)</t>
+          <t>Average community level</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad para el grifo de cocina (mg/L)</t>
+          <t>Nivel promedio de la comunidad</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Average community level for kitchen tap (μg/L)</t>
+          <t>Average community level (NTU)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad para el grifo de cocina (μg/L)</t>
+          <t>Nivel promedio de la comunidad (NTU)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Average community level measures</t>
+          <t>Average community level (mg/L)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Medidas promedios de la comunidad</t>
+          <t>Nivel promedio de la comunidad (mg/L)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Average community levels for kitchen tap</t>
+          <t>Average community level (μg/L)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Nivel promedio de la comunidad para el grifo de cocina</t>
+          <t>Nivel comunitario promedio (μg/L)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Avoid internal plumbing influence</t>
+          <t>Average community level for kitchen tap</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Evitar la influencia de la plomería interna</t>
+          <t>Nivel promedio de la comunidad para el grifo de cocina</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Avoid the influence of internal plumbing</t>
+          <t>Average community level for kitchen tap (NTU)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Eviten la influencia de la plomería interna</t>
+          <t>Nivel promedio de la comunidad para cocina de cocina (NTU)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Bacteria</t>
+          <t>Average community level for kitchen tap (mg/L)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Bacterias</t>
+          <t>Nivel promedio de la comunidad para el grifo de cocina (mg/L)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Bacteria (E. Coli)</t>
+          <t>Average community level for kitchen tap (μg/L)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Bacterias (E. Coli)</t>
+          <t>Nivel promedio de la comunidad para el grifo de cocina (μg/L)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Bad smell</t>
+          <t>Average community level measures</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Mal olor</t>
+          <t>Medidas promedios de la comunidad</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Bad taste</t>
+          <t>Average community levels for kitchen tap</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Mal sabor</t>
+          <t>Nivel promedio de la comunidad para el grifo de cocina</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Bottled water is usually regulated and must meet quality standards set by government agencies.</t>
+          <t>Avoid internal plumbing influence</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>El agua embotellada generalmente está regulada y sujeta a estándares de calidad establecidos por agencias.</t>
+          <t>Evitar la influencia de la plomería interna</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>By examining both samples, we can better understand how water usage in your home, as well as your plumbing and filtration system (if any), impact your household's water quality.</t>
+          <t>Avoid the influence of internal plumbing</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Al examinar ambas muestras, podemos comprender mejor cómo el uso del agua en su hogar, así como su sistema de plomería y filtración (si corresponde), impactan la calidad del agua de su hogar.</t>
+          <t>Eviten la influencia de la plomería interna</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Chloramine</t>
+          <t>Bacteria</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Cloramina</t>
+          <t>Bacterias</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Choosing Home Water Filters &amp; Other Water Treatment Systems</t>
+          <t>Bacteria (E. Coli)</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Elegir filtros de agua en el hogar y otros sistemas de tratamiento de agua</t>
+          <t>Bacterias (E. Coli)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Choosing Home Water Filters &amp; Other Water Treatment Systems | CDC</t>
+          <t>Bad smell</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Elegir filtros de agua en el hogar y otros sistemas de tratamiento de agua | Centros para el Control y la Prevención de Enfermedades</t>
+          <t>Mal olor</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Click here to watch our video guide. It will help you understand and use this report better.</t>
+          <t>Bad taste</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Haz clic aquí para ver nuestra guía en video. Le ayudará a comprender y utilizar mejor este informe.</t>
+          <t>Mal sabor</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Clickable report</t>
+          <t>Bottled water is usually regulated and must meet quality standards set by government agencies.</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Informe en el que se puede hacer clic</t>
+          <t>El agua embotellada generalmente está regulada y sujeta a estándares de calidad establecidos por agencias.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Cloudy water or visible particles</t>
+          <t>By examining both samples, we can better understand how water usage in your home, as well as your plumbing and filtration system (if any), impact your household's water quality.</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Agua turbia o partículas visibles</t>
+          <t>Al examinar ambas muestras, podemos comprender mejor cómo el uso del agua en su hogar, así como su sistema de plomería y filtración (si corresponde), impactan la calidad del agua de su hogar.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Concerns and questions</t>
+          <t>Chloramine</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Preocupaciones y preguntas</t>
+          <t>Cloramina</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Contact Texas Commission on Environmental Quality (TCEQ)</t>
+          <t>Choosing Home Water Filters &amp; Other Water Treatment Systems</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Comuníquese con La Comisión de Calidad Ambiental de Texas (TCEQ)</t>
+          <t>Elegir filtros de agua en el hogar y otros sistemas de tratamiento de agua</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Contact WCWH</t>
+          <t>Choosing Home Water Filters &amp; Other Water Treatment Systems | CDC</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Contactar a NCNS</t>
+          <t>Elegir filtros de agua en el hogar y otros sistemas de tratamiento de agua | Centros para el Control y la Prevención de Enfermedades</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Contact your water utility</t>
+          <t>City of Kyle</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Comuníquese con su empresa suministradora de agua</t>
+          <t>ciudad de kyle</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>County Line SUD</t>
+          <t>City of Manor</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Línea del condado SUD</t>
+          <t>ciudad de mansión</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Date of water sample</t>
+          <t>Click here to watch our video guide. It will help you understand and use this report better.</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Fecha de la muestra de agua</t>
+          <t>Haz clic aquí para ver nuestra guía en video. Le ayudará a comprender y utilizar mejor este informe.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Date of water sample: 07/26/2025</t>
+          <t>Clickable report</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Fecha de muestra de agua: 26/07/2025</t>
+          <t>Informe en el que se puede hacer clic</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Date of water sample: 09/07/2024</t>
+          <t>Cloudy water or visible particles</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Fecha de muestra de agua: 07/09/2024</t>
+          <t>Agua turbia o partículas visibles</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Date of water sample: 10/07/2024</t>
+          <t>Concerns and questions</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Fecha de muestra de agua: 10/07/2024</t>
+          <t>Preocupaciones y preguntas</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Date of water sample: 11/01/2024</t>
+          <t>Contact Texas Commission on Environmental Quality (TCEQ)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Fecha de muestra de agua: 11/01/2024</t>
+          <t>Comuníquese con La Comisión de Calidad Ambiental de Texas (TCEQ)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Date of water sample: 11/05/2025</t>
+          <t>Contact WCWH</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Fecha de la muestra de agua: 05/11/2025</t>
+          <t>Contactar a NCNS</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Detailed Test Results</t>
+          <t>Contact your water utility</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Resultados detallados de la prueba</t>
+          <t>Comuníquese con su empresa suministradora de agua</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2023.</t>
+          <t>County Line SUD</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>¿Sabía que su empresa de servicios de agua emite un informe anual de calidad del agua? Puede hacer clic en el texto naranja abajo para obtener el informe de calidad de agua de su utilidad de agua. Este informe muestra que su utilidad de agua ha cumplido con los estándares de calidad del agua requeridos del gobierno. El informe se basa en muestras recolectadas en toda el área en 2023.</t>
+          <t>Línea del condado SUD</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2024.</t>
+          <t>Date of water sample</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>¿Sabía que su empresa de servicios de agua emite un informe anual sobre la calidad del agua? Puede hacer clic en el texto naranja para obtener el informe de calidad del agua de su empresa de agua. Este informe muestra que su empresa de agua ha cumplido con los estándares de calidad del agua requeridos por el gobierno. El informe se basa en muestras recolectadas en toda el área en 2024.</t>
+          <t>Fecha de la muestra de agua</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2024. Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
+          <t>Date of water sample: 01/15/2025</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>¿Sabía que su empresa de servicios de agua emite un informe anual sobre la calidad del agua? Puede hacer clic en el texto naranja para obtener el informe de calidad del agua de su empresa de agua. Este informe muestra que su empresa de agua ha cumplido con los estándares de calidad del agua requeridos por el gobierno. El informe se basa en muestras recolectadas en toda el área en 2024. Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
+          <t>Fecha de la muestra de agua: 15/01/2025</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2025.</t>
+          <t>Date of water sample: 07/26/2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>¿Sabía que su empresa de servicios de agua emite un informe anual sobre la calidad del agua? Puede hacer clic en el texto naranja para obtener el informe de calidad del agua de su empresa de agua. Este informe muestra que su empresa de agua ha cumplido con los estándares de calidad del agua requeridos por el gobierno. El informe se basa en muestras recolectadas en toda el área en 2025.</t>
+          <t>Fecha de muestra de agua: 26/07/2025</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Did you know your water utility company issues a yearly water quality report? You can click on the text in the orange button to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2023.</t>
+          <t>Date of water sample: 09/07/2024</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>¿Sabía que su empresa de servicios de agua emite un informe anual de calidad del agua? Puede hacer clic en el texto del botón naranja para obtener el informe de calidad de agua de su utilidad de agua. Este informe muestra que su utilidad de agua ha cumplido con los estándares de calidad del agua requeridos del gobierno. El informe se basa en muestras recolectadas en toda el área en 2023.</t>
+          <t>Fecha de muestra de agua: 07/09/2024</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Discover the results of Whole Communities-Whole Health's latest water testing endeavors in your house and neighborhood. By prioritizing waterquality, we foster a healthier environment and a more resilient community.</t>
+          <t>Date of water sample: 10/07/2024</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Descubra los resultados de los últimos esfuerzos de análisis de agua de Nuestra Comunidad-Nuestra Salud en su casa y vecindario. Al priorizar la calidad del agua, fomentamos un medio ambiente más saludable y una comunidad más resiliente.</t>
+          <t>Fecha de muestra de agua: 10/07/2024</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Disinfectant</t>
+          <t>Date of water sample: 11/01/2024</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Desinfectante</t>
+          <t>Fecha de muestra de agua: 11/01/2024</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Disinfectant is added at the treatment plant to control the growth of bacteria and viruses in the water. It helps ensure that the water reaching your house is safe to drink. Low levels of disinfectant should be present in the water to maintain its safety.</t>
+          <t>Date of water sample: 11/05/2025</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Se añade desinfectante en la planta de tratamiento para controlar el crecimiento de bacterias y virus en el agua. Esto ayuda a garantizar que el agua que llega a su hogar sea segura para el consumo. Para mantener su seguridad, deben mantenerse bajos niveles de desinfectante en el agua.</t>
+          <t>Fecha de la muestra de agua: 05/11/2025</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Disinfectant: Free chlorine OR Chloramine</t>
+          <t>Detailed Test Results</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Desinfectante: cloro libre O cloramina</t>
+          <t>Resultados detallados de la prueba</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Distribution of WCWH water samples and their water utilities</t>
+          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2023.</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Distribución de muestras de agua de NCNS y sus servicios de agua</t>
+          <t>¿Sabía que su empresa de servicios de agua emite un informe anual de calidad del agua? Puede hacer clic en el texto naranja abajo para obtener el informe de calidad de agua de su utilidad de agua. Este informe muestra que su utilidad de agua ha cumplido con los estándares de calidad del agua requeridos del gobierno. El informe se basa en muestras recolectadas en toda el área en 2023.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Distribution of WCWH water samples by utility and water source</t>
+          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2024.</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Distribución de las muestras de agua de NCNS por compañía de servicio y fuente de agua</t>
+          <t>¿Sabía que su empresa de servicios de agua emite un informe anual sobre la calidad del agua? Puede hacer clic en el texto naranja para obtener el informe de calidad del agua de su empresa de agua. Este informe muestra que su empresa de agua ha cumplido con los estándares de calidad del agua requeridos por el gobierno. El informe se basa en muestras recolectadas en toda el área en 2024.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Drink bottled water</t>
+          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2024. Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Beber agua embotellada</t>
+          <t>¿Sabía que su empresa de servicios de agua emite un informe anual sobre la calidad del agua? Puede hacer clic en el texto naranja para obtener el informe de calidad del agua de su empresa de agua. Este informe muestra que su empresa de agua ha cumplido con los estándares de calidad del agua requeridos por el gobierno. El informe se basa en muestras recolectadas en toda el área en 2024. Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Drinking Water Regulations by US EPA</t>
+          <t>Did you know your water utility company issues a yearly water quality report? You can click on the orange text to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2025.</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Regulaciones del Agua Potable</t>
+          <t>¿Sabía que su empresa de servicios de agua emite un informe anual sobre la calidad del agua? Puede hacer clic en el texto naranja para obtener el informe de calidad del agua de su empresa de agua. Este informe muestra que su empresa de agua ha cumplido con los estándares de calidad del agua requeridos por el gobierno. El informe se basa en muestras recolectadas en toda el área en 2025.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Drinking water distribution system</t>
+          <t>Did you know your water utility company issues a yearly water quality report? You can click on the text in the orange button to get your water utility's water quality report. This report shows that your water utility has met the government's required water quality standards. The report is based on samples collected throughout the area in 2023.</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sistema de distribución de agua potable</t>
+          <t>¿Sabía que su empresa de servicios de agua emite un informe anual de calidad del agua? Puede hacer clic en el texto del botón naranja para obtener el informe de calidad de agua de su utilidad de agua. Este informe muestra que su utilidad de agua ha cumplido con los estándares de calidad del agua requeridos del gobierno. El informe se basa en muestras recolectadas en toda el área en 2023.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>E. coli is a sign that there might be fecal contamination. This means there could be waste or sewage in the water, which can be dangerous for your health.</t>
+          <t>Discover the results of Whole Communities-Whole Health's latest water testing endeavors in your house and neighborhood. By prioritizing waterquality, we foster a healthier environment and a more resilient community.</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>La E. coli es un indicio de que podría haber contaminación fecal. Esto significa que podría haber desechos o aguas residuales en el agua, lo cual puede ser peligroso para su salud.</t>
+          <t>Descubra los resultados de los últimos esfuerzos de análisis de agua de Nuestra Comunidad-Nuestra Salud en su casa y vecindario. Al priorizar la calidad del agua, fomentamos un medio ambiente más saludable y una comunidad más resiliente.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>El filtro en el grifo de la cocina elimina el cloro, que está previsto. Esto no es un problema ya que no hay suficiente tiempo para que crezcan bacterias dañinas. Las concentraciones del cloro en interiores y exteriores demuestran que el cloro está siendo entregado a su hogar, eliminando las bacterias dañinas en su suministro de agua.</t>
+          <t>Disinfectant</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>El filtro en el grifo de la cocina elimina el cloro que está previsto. Esto no es un problema ya que no hay tiempo suficiente para que crezcan bacterias dañinas. Las concentraciones del cloro en interiores y exteriores demuestran que el cloro está siendo entregado a su hogar, eliminando las bacterias dañinas en su suministro de agua.</t>
+          <t>Desinfectante</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Filtered drinking water</t>
+          <t>Disinfectant is added at the treatment plant to control the growth of bacteria and viruses in the water. It helps ensure that the water reaching your house is safe to drink. Low levels of disinfectant should be present in the water to maintain its safety.</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Su agua potable filtrada</t>
+          <t>Se añade desinfectante en la planta de tratamiento para controlar el crecimiento de bacterias y virus en el agua. Esto ayuda a garantizar que el agua que llega a su hogar sea segura para el consumo. Para mantener su seguridad, deben mantenerse bajos niveles de desinfectante en el agua.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>For example, the quality of water that water utilities supply to households should be better than the quality of the water in lakes and streams.</t>
+          <t>Disinfectant: Free chlorine OR Chloramine</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Por ejemplo, la calidad del agua que los servicios de agua suministran a los hogares debe ser mejor que la calidad del agua de lagos y arroyos.</t>
+          <t>Desinfectante: cloro libre O cloramina</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Free chlorine</t>
+          <t>Distribution of WCWH water samples and their water utilities</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Cloro libre</t>
+          <t>Distribución de muestras de agua de NCNS y sus servicios de agua</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Glossary</t>
+          <t>Distribution of WCWH water samples by utility and water source</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Glosario</t>
+          <t>Distribución de las muestras de agua de NCNS por compañía de servicio y fuente de agua</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Hardness</t>
+          <t>Drink bottled water</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>La dureza del agua</t>
+          <t>Beber agua embotellada</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Drinking Water Regulations by US EPA</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Altos</t>
+          <t>Regulaciones del Agua Potable</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>High lead levels can cause harmful health effects, especially for pregnant women and young children.</t>
+          <t>Drinking water distribution system</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Los niveles altos de plomo pueden causar efectos perjudiciales para la salud, especialmente para las mujeres embarazadas y los niños pequeños.</t>
+          <t>Sistema de distribución de agua potable</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>High levels of these substances can harm your health.</t>
+          <t>E. coli is a sign that there might be fecal contamination. This means there could be waste or sewage in the water, which can be dangerous for your health.</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Altos niveles de estas sustancias pueden perjudicar su salud.</t>
+          <t>La E. coli es un indicio de que podría haber contaminación fecal. Esto significa que podría haber desechos o aguas residuales en el agua, lo cual puede ser peligroso para su salud.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>High turbidity will give water a cloudy appearance. This does not mean the water is unsafe necessarily, but could indicate the water has become contaminated.</t>
+          <t>El filtro en el grifo de la cocina elimina el cloro, que está previsto. Esto no es un problema ya que no hay suficiente tiempo para que crezcan bacterias dañinas. Las concentraciones del cloro en interiores y exteriores demuestran que el cloro está siendo entregado a su hogar, eliminando las bacterias dañinas en su suministro de agua.</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Una alta turbidez dará al agua una apariencia turbia. Esto no significa necesariamente que el agua sea insegura, pero podría indicar que el agua se ha contaminado.</t>
+          <t>El filtro en el grifo de la cocina elimina el cloro que está previsto. Esto no es un problema ya que no hay tiempo suficiente para que crezcan bacterias dañinas. Las concentraciones del cloro en interiores y exteriores demuestran que el cloro está siendo entregado a su hogar, eliminando las bacterias dañinas en su suministro de agua.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Home plumbing and filtration systems</t>
+          <t>Filtered drinking water</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Sistemas de filtración y cañería del hogar</t>
+          <t>Su agua potable filtrada</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Hornsense ID: WC0019</t>
+          <t>For example, the quality of water that water utilities supply to households should be better than the quality of the water in lakes and streams.</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>ID de Hornsense: WC0019</t>
+          <t>Por ejemplo, la calidad del agua que los servicios de agua suministran a los hogares debe ser mejor que la calidad del agua de lagos y arroyos.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Hornsense ID: WC0156</t>
+          <t>Free chlorine</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>ID de Hornsense: WC0156</t>
+          <t>Cloro libre</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Hornsense ID: WC6449</t>
+          <t>Glossary</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>ID de Hornsense: WC6449</t>
+          <t>Glosario</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Hornsense ID: WC7755</t>
+          <t>Hardness</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>ID de Hornsense: WC7755</t>
+          <t>La dureza del agua</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Hornsense ID: WC8120</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>ID de Hornsense: WC8120</t>
+          <t>Altos</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Hose tap immediately outside your home after flushing the water line</t>
+          <t>High lead levels can cause harmful health effects, especially for pregnant women and young children.</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Grifo de manguera inmediatamente afuera de su hogar después de descargar la línea.</t>
+          <t>Los niveles altos de plomo pueden causar efectos perjudiciales para la salud, especialmente para las mujeres embarazadas y los niños pequeños.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>How to read your results</t>
+          <t>High levels of these substances can harm your health.</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Cómo leer sus resultados</t>
+          <t>Altos niveles de estas sustancias pueden perjudicar su salud.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>If you are worried about the safety of your drinking water, there are some temporary actions you can take while your water is being checked.</t>
+          <t>High turbidity will give water a cloudy appearance. This does not mean the water is unsafe necessarily, but could indicate the water has become contaminated.</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Si le preocupa la seguridad de su agua potable, hay algunas acciones que puede tomar temporalmente mientras se investiga su agua.</t>
+          <t>Una alta turbidez dará al agua una apariencia turbia. Esto no significa necesariamente que el agua sea insegura, pero podría indicar que el agua se ha contaminado.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>If you have concerns about water quality...</t>
+          <t>Home plumbing and filtration systems</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Si tiene dudas sobre la calidad del agua…</t>
+          <t>Sistemas de filtración y cañería del hogar</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>If you have concerns, you can report the problem anonymously or leave your name and contact information.</t>
+          <t>Hornsense ID: MOCK-P9103T</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Si tiene dudas, puede informar el problema de forma anónima o dejar su nombre e información de contacto.</t>
+          <t>Identificación de Hornsense: MOCK-P9103T</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>If you think your water has major problems, contact your water utility. They will collect a water sample from your house for testing.</t>
+          <t>Hornsense ID: MOCK-P9104T</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Si sospecha que su agua tiene problemas importantes, debe comunicarse con la empresa suministradora de agua. Existen laboratorios certificados que pueden analizar su agua.</t>
+          <t>Identificación de Hornsense: MOCK-P9104T</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Important Note</t>
+          <t>Hornsense ID: WC0019</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Nota importante</t>
+          <t>ID de Hornsense: WC0019</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Important note</t>
+          <t>Hornsense ID: WC0156</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Nota importante</t>
+          <t>ID de Hornsense: WC0156</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>In acceptable range</t>
+          <t>Hornsense ID: WC6449</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>En rango aceptable</t>
+          <t>ID de Hornsense: WC6449</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>In agreement with your Utility Company Report</t>
+          <t>Hornsense ID: WC7755</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>De acuerdo con su Informe de Empresa de Servicios Públicos</t>
+          <t>ID de Hornsense: WC7755</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>In normal range</t>
+          <t>Hornsense ID: WC8120</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>En rango normal</t>
+          <t>ID de Hornsense: WC8120</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>In our study, WCWH participants expressed a desire to know more about the quality of the water in their homes.</t>
+          <t>Hose tap immediately outside your home after flushing the water line</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>En nuestro estudio, los participantes de NCNS expresaron su deseo de saber más sobre la calidad del agua de sus hogares.</t>
+          <t>Grifo de manguera inmediatamente afuera de su hogar después de descargar la línea.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Indoor</t>
+          <t>How to read your results</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Interior</t>
+          <t>Cómo leer sus resultados</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Indoor water quality measures</t>
+          <t>If you are worried about the safety of your drinking water, there are some temporary actions you can take while your water is being checked.</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Medidas de calidad del agua en interiores</t>
+          <t>Si le preocupa la seguridad de su agua potable, hay algunas acciones que puede tomar temporalmente mientras se investiga su agua.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>It's important to stay aware of your water quality because it can change over time. Look out for these signs of potential problems:</t>
+          <t>If you have concerns about water quality...</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Es importante estar al tanto de la calidad de su agua porque puede cambiar con el tiempo. Esté atento a estas señales de posibles problemas:</t>
+          <t>Si tiene dudas sobre la calidad del agua…</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Kitchen faucet inside your home after flushing the water line.</t>
+          <t>If you have concerns, you can report the problem anonymously or leave your name and contact information.</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Grifo dentro de su hogar después de descargar la línea.</t>
+          <t>Si tiene dudas, puede informar el problema de forma anónima o dejar su nombre e información de contacto.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Know more about commercially bottled water</t>
+          <t>If you think your water has major problems, contact your water utility. They will collect a water sample from your house for testing.</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Conoce más sobre el agua embotellada comercialmente</t>
+          <t>Si sospecha que su agua tiene problemas importantes, debe comunicarse con la empresa suministradora de agua. Existen laboratorios certificados que pueden analizar su agua.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>L: liter</t>
+          <t>Important Note</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>L: litro</t>
+          <t>Nota importante</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Important note</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Plomo</t>
+          <t>Nota importante</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Learn About Your Report</t>
+          <t>In acceptable range</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Más información sobre su informe</t>
+          <t>En rango aceptable</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>In agreement with your Utility Company Report</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Bajos</t>
+          <t>De acuerdo con su Informe de Empresa de Servicios Públicos</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>In normal range</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>En rango normal</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Meet regulatory guidelines</t>
+          <t>In our study, WCWH participants expressed a desire to know more about the quality of the water in their homes.</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Cumplen con las directrices regulatorias</t>
+          <t>En nuestro estudio, los participantes de NCNS expresaron su deseo de saber más sobre la calidad del agua de sus hogares.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Meets the standards established by the Texas Commission on Environmental Quality.</t>
+          <t>Indoor</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Cumple con los estándares establecidos por la Comisión de Calidad Ambiental de Texas.</t>
+          <t>Interior</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Met governmental standards</t>
+          <t>Indoor water quality measures</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Cumplió con los estándares gubernamentales</t>
+          <t>Medidas de calidad del agua en interiores</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Met governmental standards?</t>
+          <t>It's important to stay aware of your water quality because it can change over time. Look out for these signs of potential problems:</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>¿Cumplió con los estándares gubernamentales?</t>
+          <t>Es importante estar al tanto de la calidad de su agua porque puede cambiar con el tiempo. Esté atento a estas señales de posibles problemas:</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Minimize contamination</t>
+          <t>Kitchen faucet inside your home after flushing the water line.</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Minimizan la contaminación</t>
+          <t>Grifo dentro de su hogar después de descargar la línea.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>NTU: Nephelometric Turbidity Unit</t>
+          <t>Know more about commercially bottled water</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>NTU: Unidad Nefelométrica de Turbidez</t>
+          <t>Conoce más sobre el agua embotellada comercialmente</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Nitrate</t>
+          <t>L: liter</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Nitrato</t>
+          <t>L: litro</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Nitrite</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Nitrito</t>
+          <t>Plomo</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Learn About Your Report</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Más información sobre su informe</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>No regulated standard</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Sin estándar regulado</t>
+          <t>Bajos</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Not detected</t>
+          <t>Manor City Hall 105 E. Eggleston St.</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>No detectado</t>
+          <t>Ayuntamiento de Manor 105 E. Eggleston St.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Official Website</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Sitio web oficial</t>
+          <t>Moderado</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Online Report Portal</t>
+          <t>Meet regulatory guidelines</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Portal de informes</t>
+          <t>Cumplen con las directrices regulatorias</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Out of acceptable range</t>
+          <t>Meets the standards established by the Texas Commission on Environmental Quality.</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Fuera del rango aceptable</t>
+          <t>Cumple con los estándares establecidos por la Comisión de Calidad Ambiental de Texas.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Out of normal range</t>
+          <t>Met governmental standards</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Fuera del rango normal</t>
+          <t>Cumplió con los estándares gubernamentales</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Outdoor</t>
+          <t>Met governmental standards?</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Exterior</t>
+          <t>¿Cumplió con los estándares gubernamentales?</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Outdoor water quality measures</t>
+          <t>Minimize contamination</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Medidas de calidad del agua al aire libre</t>
+          <t>Minimizan la contaminación</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
+          <t>NTU: Nephelometric Turbidity Unit</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
+          <t>NTU: Unidad Nefelométrica de Turbidez</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Parameters' snapshot</t>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Resumen de los resultados de la prueba</t>
+          <t>Nitrato</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Potential source and meaning</t>
+          <t>Nitrite</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Fuentes potenciales / Significado</t>
+          <t>Nitrito</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Presence of E. coli can cause sickness.</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>La presencia de E. coli puede causar enfermedades.</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Produced by WCWH</t>
+          <t>No regulated standard</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Producido por NCNS</t>
+          <t>Sin estándar regulado</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Report any water quality issues in the WCWH app</t>
+          <t>Not detected</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Utilice la aplicación de NCNS para informar cualquier problema con la calidad del agua</t>
+          <t>No detectado</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Report your concern</t>
+          <t>Official Website</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Informar inquietudes</t>
+          <t>Sitio web oficial</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Represent your water supply</t>
+          <t>Online Report Portal</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Representan su suministro de agua</t>
+          <t>Portal de informes</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Return to table of contents</t>
+          <t>Out of acceptable range</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Volver a la tabla de contenidos</t>
+          <t>Fuera del rango aceptable</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Runoff from fertilizer use; leaching from septic tanks, sewage.</t>
+          <t>Out of normal range</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Escorrentía de uso de fertilizantes; lixiviación de tanques sépticos, aguas residuales.</t>
+          <t>Fuera del rango normal</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Sampled by utilities</t>
+          <t>Outdoor</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Muestreado por utilidades</t>
+          <t>Exterior</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Samples were collected from:</t>
+          <t>Outdoor water quality measures</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Muestra recogida de:</t>
+          <t>Medidas de calidad del agua al aire libre</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
+          <t>Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Para asistencia en español, favor de llamar al teléfono (512) 304-0354.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Parameters' snapshot</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Resumen de los resultados de la prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Potential source and meaning</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Fuentes potenciales / Significado</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Presence of E. coli can cause sickness.</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>La presencia de E. coli puede causar enfermedades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Produced by WCWH</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Producido por NCNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Report any water quality issues in the WCWH app</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Utilice la aplicación de NCNS para informar cualquier problema con la calidad del agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Report your concern</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Informar inquietudes</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Represent your water supply</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Representan su suministro de agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Return to table of contents</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Volver a la tabla de contenidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Runoff from fertilizer use; leaching from septic tanks, sewage.</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Escorrentía de uso de fertilizantes; lixiviación de tanques sépticos, aguas residuales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Sampled by utilities</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Muestreado por utilidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Samples were collected from:</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Muestra recogida de:</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
           <t>Several factors can influence the quality of the drinking water
               supplied to your home. These factors include:</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr">
+      <c r="B183" t="inlineStr">
         <is>
           <t>Varios factores pueden influir en la calidad del agua potable.
               suministrado a su hogar. Estos factores incluyen:</t>
         </is>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>Several factors can influence the quality of the drinking water supplied to your home. These factors include:</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>Hay varios factores que pueden influir en la calidad del agua potable suministrada a su hogar. Estos factores incluyen:</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>Since the tests we did were within the governmental standards</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>Dado que las pruebas que realizamos estaban dentro de los estándares gubernamentales:</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>Some plumbing systems, like pipes and fixtures, are made of lead. When these corrode, they can increase the levels of lead in drinking water.</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>Algunos sistemas de plomería, como las tuberías y accesorios, están hechos de plomo. Cuando estos se corroen, pueden aumentar los niveles de plomo en el agua potable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>Source of water</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>Origen del agua</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>Stay aware of your water quality</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>Manténgase alerta sobre la calidad del agua</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>TCEQ</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>TCEQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>TCEQ has set standards for drinking water quality</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>La Comisión de Calidad Ambiental de Texas (TCEQ) ha establecido estándares para la calidad del agua potable</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>Table Of Contents</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>Tabla de contenidos</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>Talk to your neighbors</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>Hable con sus vecinos</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>Talk to your neighbors to see if they have similar concerns.</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Hable con sus vecinos para ver si tienen preocupaciones similares.</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>Temporary solutions</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>Soluciones temporales</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>Test Results Overview</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Resumen de los resultados de la prueba</t>
-        </is>
-      </c>
-    </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>The EPA has legal limits for over 90 contaminants. Whole Communities-Whole Health tests for 7 contaminants in drinking water because of time and cost.</t>
+          <t>Several factors can influence the quality of the drinking water supplied to your home. These factors include:</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>La EPA tiene límites legales para más de 90 contaminantes. NCNS analiza 7 contaminantes en el agua potable debido a limitaciones de tiempo y costo.</t>
+          <t>Hay varios factores que pueden influir en la calidad del agua potable suministrada a su hogar. Estos factores incluyen:</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>The EPA has legal limits for over 90 parameters. Whole Communities-Whole Health tests for 7 parameters in drinking water because of time and cost.</t>
+          <t>Since the tests we did were within the governmental standards</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>La EPA tiene límites legales para más de 90 parámetros. NCNS analiza 7 parámetros en el agua potable debido a limitaciones de tiempo y costo.</t>
+          <t>Dado que las pruebas que realizamos estaban dentro de los estándares gubernamentales:</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>The EPA has legal limits for over 90 parameters. Whole Communities-Whole Health tests for 8 parameters in drinking water because of time and cost.</t>
+          <t>Some plumbing systems, like pipes and fixtures, are made of lead. When these corrode, they can increase the levels of lead in drinking water.</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>La EPA tiene límites legales para más de 90 parámetros. Comunidades enteras: las pruebas de salud de todo el mundo para 8 parámetros en el agua potable debido al tiempo y el costo.</t>
+          <t>Algunos sistemas de plomería, como las tuberías y accesorios, están hechos de plomo. Cuando estos se corroen, pueden aumentar los niveles de plomo en el agua potable.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>The Texas Commission on Environmental Quality (TCEQ) and the Environmental Protection Agency (EPA) have set standards for drinking water quality. All water treatment plants in Texas must meet these standards.</t>
+          <t>Source of water</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>La Comisión de Calidad Ambiental de Texas (TCEQ) y la Agencia de Protección Ambiental (EPA) han establecido estándares para la calidad del agua potable ​​​​que todos los sistemas de tratamiento de agua en Texas deben cumplir.</t>
+          <t>Origen del agua</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>The WCWH test is based on 7 parameters:</t>
+          <t>Stay aware of your water quality</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>La prueba WCWH se basa en 7 parámetros:</t>
+          <t>Manténgase alerta sobre la calidad del agua</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>The WCWH test is based on 8 parameters:</t>
+          <t>TCEQ</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>La prueba WCWH se basa en 8 parámetros:</t>
+          <t>TCEQ</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>The figures below show the distribution of homes sampled by their water utility and where those utilities source their water.</t>
+          <t>TCEQ has set standards for drinking water quality</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Las cifras a continuación muestran la distribución de casas muestreadas por su utilidad de agua y donde esas empresas de servicios públicos obtienen su agua.</t>
+          <t>La Comisión de Calidad Ambiental de Texas (TCEQ) ha establecido estándares para la calidad del agua potable</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>The network of pipes that carry water to your home can have an impact on its quality.</t>
+          <t>Table Of Contents</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>La red de tuberías que transportan el agua a su hogar puede influir su calidad.</t>
+          <t>Tabla de contenidos</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>The plumbing in your home and any installed water filtration systems can influence the water quality.</t>
+          <t>Talk to your neighbors</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>La cañería de su hogar y cualquier sistema de filtración de agua instalado pueden influir en la calidad del agua.</t>
+          <t>Hable con sus vecinos</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>The quality of the water in your home can vary based on the amount of water you use and the timing of when you use it.</t>
+          <t>Talk to your neighbors to see if they have similar concerns.</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>La calidad del agua de su hogar puede variar en función de la cantidad de agua que utilice y del momento en que la utilice.</t>
+          <t>Hable con sus vecinos para ver si tienen preocupaciones similares.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>The test is a spot check</t>
+          <t>Temporary solutions</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>La prueba es una verificación puntual</t>
+          <t>Soluciones temporales</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>The water in your home typically comes from a lake, river, or groundwater source.</t>
+          <t>Test Results Overview</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>El agua de su hogar suele proceder de un lago, un río o una fuente subterránea.</t>
+          <t>Resumen de los resultados de la prueba</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>The way the water is treated at the treatment plant before it reaches your home can affect its quality.</t>
+          <t>The EPA has legal limits for over 90 contaminants. Whole Communities-Whole Health tests for 7 contaminants in drinking water because of time and cost.</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>La forma en que se trata el agua en la planta potabilizadora antes de que llegue a su hogar puede afectar su calidad.</t>
+          <t>La EPA tiene límites legales para más de 90 contaminantes. NCNS analiza 7 contaminantes en el agua potable debido a limitaciones de tiempo y costo.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>There is no regulated standard for this parameter</t>
+          <t>The EPA has legal limits for over 90 parameters. Whole Communities-Whole Health tests for 7 parameters in drinking water because of time and cost.</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>No hay estándar regulado para este parámetro</t>
+          <t>La EPA tiene límites legales para más de 90 parámetros. NCNS analiza 7 parámetros en el agua potable debido a limitaciones de tiempo y costo.</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>These parameters were not tested:</t>
+          <t>The EPA has legal limits for over 90 parameters. Whole Communities-Whole Health tests for 8 parameters in drinking water because of time and cost.</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Estos parámetros no fueron probados:</t>
+          <t>La EPA tiene límites legales para más de 90 parámetros. Comunidades enteras: las pruebas de salud de todo el mundo para 8 parámetros en el agua potable debido al tiempo y el costo.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>These results show the water quality at the time we took your samples. Your water quality may change over time.</t>
+          <t>The Texas Commission on Environmental Quality (TCEQ) and the Environmental Protection Agency (EPA) have set standards for drinking water quality. All water treatment plants in Texas must meet these standards.</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Estos resultados muestran la calidad del agua en el momento en que tomamos sus muestras. La calidad de su agua puede cambiar con el tiempo.</t>
+          <t>La Comisión de Calidad Ambiental de Texas (TCEQ) y la Agencia de Protección Ambiental (EPA) han establecido estándares para la calidad del agua potable ​​​​que todos los sistemas de tratamiento de agua en Texas deben cumplir.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>These sources:</t>
+          <t>The WCWH test is based on 7 parameters:</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Estas fuentes:</t>
+          <t>La prueba WCWH se basa en 7 parámetros:</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>These standards ensure that the water provided to households is treated to remove bacteria and other pollutants. Water utilities must treat drinking water to make it safe for household use.</t>
+          <t>The WCWH test is based on 8 parameters:</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Estas normas garantizan que el agua suministrada a los hogares ha sido tratada para eliminar las bacterias y otros contaminantes. Los servicios de agua están obligados a tratar el agua para que sea segura para el uso doméstico.</t>
+          <t>La prueba WCWH se basa en 8 parámetros:</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>This report does not show the complete picture of your water quality</t>
+          <t>The figures below show the distribution of homes sampled by their water utility and where those utilities source their water.</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Este informe no muestra la imagen completa de la calidad de su agua.</t>
+          <t>Las cifras a continuación muestran la distribución de casas muestreadas por su utilidad de agua y donde esas empresas de servicios públicos obtienen su agua.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>This test is a spot check</t>
+          <t>The network of pipes that carry water to your home can have an impact on its quality.</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>La prueba es una verificación puntual</t>
+          <t>La red de tuberías que transportan el agua a su hogar puede influir su calidad.</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Treatment process</t>
+          <t>The plumbing in your home and any installed water filtration systems can influence the water quality.</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Proceso de tratamiento</t>
+          <t>La cañería de su hogar y cualquier sistema de filtración de agua instalado pueden influir en la calidad del agua.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Turbidity</t>
+          <t>The quality of the water in your home can vary based on the amount of water you use and the timing of when you use it.</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Turbidez</t>
+          <t>La calidad del agua de su hogar puede variar en función de la cantidad de agua que utilice y del momento en que la utilice.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Turbidity refers to the clarity of water and the presence of particles in it. It measures how clear or cloudy the water appears.</t>
+          <t>The test is a spot check</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>La turbidez se refiere a la claridad del agua y la presencia de partículas en ella. Mide qué tan clara o turbia parece el agua.</t>
+          <t>La prueba es una verificación puntual</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Use a water filter</t>
+          <t>The water in your home typically comes from a lake, river, or groundwater source.</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Utilice un filtro de agua</t>
+          <t>El agua de su hogar suele proceder de un lago, un río o una fuente subterránea.</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>View your Annual Report here</t>
+          <t>The way the water is treated at the treatment plant before it reaches your home can affect its quality.</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Consulta su Informe Anual aquí</t>
+          <t>La forma en que se trata el agua en la planta potabilizadora antes de que llegue a su hogar puede afectar su calidad.</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>View your water utility's annual report</t>
+          <t>There is no regulated standard for this parameter</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Ver el informe anual de su empresa de agua</t>
+          <t>No hay estándar regulado para este parámetro</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>WCWH Spot Test Results</t>
+          <t>These parameters were not tested:</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Resultados de la prueba puntual de NCNS</t>
+          <t>Estos parámetros no fueron probados:</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>WCWH results of 7 measures</t>
+          <t>These results show the water quality at the time we took your samples. Your water quality may change over time.</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Resultados NCNS de 7 medidas</t>
+          <t>Estos resultados muestran la calidad del agua en el momento en que tomamos sus muestras. La calidad de su agua puede cambiar con el tiempo.</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>WCWH results of 8 measures</t>
+          <t>These sources:</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Resultados de WCWH de 8 medidas</t>
+          <t>Estas fuentes:</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Water Quality Report</t>
+          <t>These standards ensure that the water provided to households is treated to remove bacteria and other pollutants. Water utilities must treat drinking water to make it safe for household use.</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Informe de calidad del agua</t>
+          <t>Estas normas garantizan que el agua suministrada a los hogares ha sido tratada para eliminar las bacterias y otros contaminantes. Los servicios de agua están obligados a tratar el agua para que sea segura para el uso doméstico.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Water Sources</t>
+          <t>This report does not show the complete picture of your water quality</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Fuente de agua</t>
+          <t>Este informe no muestra la imagen completa de la calidad de su agua.</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Water Utilities</t>
+          <t>This test is a spot check</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Servicios de agua</t>
+          <t>La prueba es una verificación puntual</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Water is safe to drink if its pH is between 6.5 and 9.5. Water outside this range can still be safe, but it might indicate water quality problems.</t>
+          <t>Treatment process</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>El agua es segura para beber si su pH está entre 6.5 y 9.5. El agua cercana a este rango aún puede ser segura, pero podría indicar problemas en la calidad del agua.</t>
+          <t>Proceso de tratamiento</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Water quality is always changing</t>
+          <t>Turbidity</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>La calidad del agua siempre está cambiando</t>
+          <t>Turbidez</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Water quality means the condition of the water based on its chemical, physical, and biological properties. It tells us if the water is good for a specific purpose.</t>
+          <t>Turbidity refers to the clarity of water and the presence of particles in it. It measures how clear or cloudy the water appears.</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>La calidad del agua se refiere al estado del agua según sus propiedades químicas, físicas y biológicas. Nos indica si el agua es adecuada para un propósito específico.</t>
+          <t>La turbidez se refiere a la claridad del agua y la presencia de partículas en ella. Mide qué tan clara o turbia parece el agua.</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Water quality report</t>
+          <t>Use a water filter</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Informe de calidad del agua</t>
+          <t>Utilice un filtro de agua</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Water usage</t>
+          <t>View your Annual Report here</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Uso del agua</t>
+          <t>Consulta su Informe Anual aquí</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>We aim to gather information about the water quality in homes across the county and understand how it varies among different water utilities in the area.</t>
+          <t>View your water utility's annual report</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Nuestro objetivo es recopilar información sobre la calidad del agua en los hogares de todo el condado y comprender cómo varía entre los diferentes servicios de agua de la zona.</t>
+          <t>Ver el informe anual de su empresa de agua</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>We encourage you to learn more information about the contaminants on:</t>
+          <t>WCWH Spot Test Results</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Puede aprender más sobre los contaminantes en:</t>
+          <t>Resultados de la prueba puntual de NCNS</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>We encourage you to learn more information about the parameters on:</t>
+          <t>WCWH results of 7 measures</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Puede aprender más sobre los parámetros en:</t>
+          <t>Resultados NCNS de 7 medidas</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>We may not be able to respond right away, but these reports will be useful if we discuss results with water utility companies and the TCEQ (Texas Commission on Environmental Quality).</t>
+          <t>WCWH results of 8 measures</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Es posible que no podamos responder de inmediato, pero estos informes podrían ser útiles si tenemos que discutir los resultados con las empresas de agua y la TCEQ (Comisión de Calidad Ambiental de Texas).</t>
+          <t>Resultados de WCWH de 8 medidas</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>We tested your water again after one of the previous six drinking water samples taken in April 2024 came back with a high lead result. We believe this to be an error, as the other five samples at that time all had very low lead concentrations.  The new drinking water samples taken in Sepetember 2024 had very low lead concentrations as well, increasing our confidence that the one high lead sample was an error.</t>
+          <t>Water Quality Report</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Probamos su agua nuevamente después de que una de las seis muestras anteriores de agua potable tomadas en abril de 2024 regresó con un alto resultado de plomo. Creemos que esto es un error, ya que las otras cinco muestras en ese momento tenían concentraciones de plomo muy bajas.  Las nuevas muestras de agua potable tomadas en septiembre de 2024 también tuvieron concentraciones de plomo muy bajas, lo que aumentó la confianza de que la única muestra de plomo alto fue un error.</t>
+          <t>Informe de calidad del agua</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>We were unable to test for nitrite in your drinking water samples at this time.  Based on previous water samples in our Whole Community-Whole Health study we would not expect nitrite to be an issue in your drinking water.</t>
+          <t>Water Sources</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>No pudimos probar el nitrito en las muestras de agua potable en este momento.  Basado en muestras de agua anteriores en toda nuestro estudio de salud de la comunidad, no esperaríamos que el nitrito sea un problema en su agua potable.</t>
+          <t>Fuente de agua</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>What can affect the water quality in your home?</t>
+          <t>Water Utilities</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>¿Qué puede afectar la calidad del agua en su hogar?</t>
+          <t>Servicios de agua</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>What does "water quality" mean?</t>
+          <t>Water is safe to drink if its pH is between 6.5 and 9.5. Water outside this range can still be safe, but it might indicate water quality problems.</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>¿Qué significa "calidad del agua"?</t>
+          <t>El agua es segura para beber si su pH está entre 6.5 y 9.5. El agua cercana a este rango aún puede ser segura, pero podría indicar problemas en la calidad del agua.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Whole Communities-Whole Health can also make an anonymous report on your behalf if you would like</t>
+          <t>Water quality is always changing</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Si lo prefiere, NCNS puede hacer un informe anónimo en su nombre a TCEQ y/o su empresa suministradora de agua.</t>
+          <t>La calidad del agua siempre está cambiando</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Why is WCWH testing water quality?</t>
+          <t>Water quality means the condition of the water based on its chemical, physical, and biological properties. It tells us if the water is good for a specific purpose.</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>¿Por qué NCNS analiza la calidad del agua?</t>
+          <t>La calidad del agua se refiere al estado del agua según sus propiedades químicas, físicas y biológicas. Nos indica si el agua es adecuada para un propósito específico.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Why you should care</t>
+          <t>Water quality report</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>¿Por qué es importante para usted?</t>
+          <t>Informe de calidad del agua</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Water usage</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Uso del agua</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>You can click on any links and catalogs in this report. They will take you to websites or other pages in the report.</t>
+          <t>We aim to gather information about the water quality in homes across the county and understand how it varies among different water utilities in the area.</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Se puede hacer clic en todos los enlaces y catálogos para abrir sitios web o ir a las páginas correspondientes.</t>
+          <t>Nuestro objetivo es recopilar información sobre la calidad del agua en los hogares de todo el condado y comprender cómo varía entre los diferentes servicios de agua de la zona.</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>You can install filters where water enters your home or where you use it. They can remove contaminants like iron, lead, and sulfur, and also improve the taste of your water.</t>
+          <t>We encourage you to learn more information about the contaminants on:</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Los filtros se pueden instalar en el punto de entrada o punto de uso en su hogar. Pueden eliminar contaminantes como hierro, plomo y azufre, al mismo tiempo que mejoran el sabor de su agua.</t>
+          <t>Puede aprender más sobre los contaminantes en:</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>You can install filters where water enters your home or where you use it. They can remove parameters like iron, lead, and sulfur, and also improve the taste of your water.</t>
+          <t>We encourage you to learn more information about the parameters on:</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Los filtros se pueden instalar en el punto de entrada o punto de uso en su hogar. Pueden eliminar parámetros como hierro, plomo y azufre, al mismo tiempo que mejoran el sabor de su agua.</t>
+          <t>Puede aprender más sobre los parámetros en:</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>You don't need to take any action right now.</t>
+          <t>We may not be able to respond right away, but these reports will be useful if we discuss results with water utility companies and the TCEQ (Texas Commission on Environmental Quality).</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>No necesita tomar ninguna medida por ahora.</t>
+          <t>Es posible que no podamos responder de inmediato, pero estos informes podrían ser útiles si tenemos que discutir los resultados con las empresas de agua y la TCEQ (Comisión de Calidad Ambiental de Texas).</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
+          <t>We tested your water again after one of the previous six drinking water samples taken in April 2024 came back with a high lead result. We believe this to be an error, as the other five samples at that time all had very low lead concentrations.  The new drinking water samples taken in Sepetember 2024 had very low lead concentrations as well, increasing our confidence that the one high lead sample was an error.</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Probamos su agua nuevamente después de que una de las seis muestras anteriores de agua potable tomadas en abril de 2024 regresó con un alto resultado de plomo. Creemos que esto es un error, ya que las otras cinco muestras en ese momento tenían concentraciones de plomo muy bajas.  Las nuevas muestras de agua potable tomadas en septiembre de 2024 también tuvieron concentraciones de plomo muy bajas, lo que aumentó la confianza de que la única muestra de plomo alto fue un error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>We were unable to test for nitrite in your drinking water samples at this time.  Based on previous water samples in our Whole Community-Whole Health study we would not expect nitrite to be an issue in your drinking water.</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>No pudimos probar el nitrito en las muestras de agua potable en este momento.  Basado en muestras de agua anteriores en toda nuestro estudio de salud de la comunidad, no esperaríamos que el nitrito sea un problema en su agua potable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>What can affect the water quality in your home?</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>¿Qué puede afectar la calidad del agua en su hogar?</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>What does "water quality" mean?</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>¿Qué significa "calidad del agua"?</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Whole Communities-Whole Health can also make an anonymous report on your behalf if you would like</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Si lo prefiere, NCNS puede hacer un informe anónimo en su nombre a TCEQ y/o su empresa suministradora de agua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Why is WCWH testing water quality?</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>¿Por qué NCNS analiza la calidad del agua?</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Why you should care</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>¿Por qué es importante para usted?</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>You can click on any links and catalogs in this report. They will take you to websites or other pages in the report.</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Se puede hacer clic en todos los enlaces y catálogos para abrir sitios web o ir a las páginas correspondientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>You can install filters where water enters your home or where you use it. They can remove contaminants like iron, lead, and sulfur, and also improve the taste of your water.</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Los filtros se pueden instalar en el punto de entrada o punto de uso en su hogar. Pueden eliminar contaminantes como hierro, plomo y azufre, al mismo tiempo que mejoran el sabor de su agua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>You can install filters where water enters your home or where you use it. They can remove parameters like iron, lead, and sulfur, and also improve the taste of your water.</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Los filtros se pueden instalar en el punto de entrada o punto de uso en su hogar. Pueden eliminar parámetros como hierro, plomo y azufre, al mismo tiempo que mejoran el sabor de su agua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>You don't need to take any action right now.</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>No necesita tomar ninguna medida por ahora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
           <t>Your Water Utility's Annual
               Report</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr">
+      <c r="B249" t="inlineStr">
         <is>
           <t>El servicio anual de su servicio de agua
               Informe</t>
         </is>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>Your Water Utility's Annual Report</t>
-        </is>
-      </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>Informe Anual de Su Proveedor de Agua</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>Your filtered drinking water</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>Su agua potable filtrada</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>Your filtered drinking water (NTU)</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>Su agua potable filtrada (NTU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>Your filtered drinking water (mg/L)</t>
-        </is>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>Su agua potable filtrada (mg/L)</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="inlineStr">
-        <is>
-          <t>Your filtered drinking water (μg/L)</t>
-        </is>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>Su agua potable filtrada (μg/L)</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>Your kitchen tap</t>
-        </is>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>Su grifo de cocina</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="inlineStr">
-        <is>
-          <t>Your kitchen tap (NTU)</t>
-        </is>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>Su grifo de cocina (ntu)</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="inlineStr">
-        <is>
-          <t>Your kitchen tap (mg/L)</t>
-        </is>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>Su grifo de cocina (mg/L)</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>Your kitchen tap (μg/L)</t>
-        </is>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>Su grifo de cocina (μg/L)</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="inlineStr">
-        <is>
-          <t>Your level</t>
-        </is>
-      </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>Su nivel</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="inlineStr">
-        <is>
-          <t>Your level (NTU)</t>
-        </is>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>Su nivel (NTU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>Your level (mg/L)</t>
-        </is>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>Su nivel (mg/L)</t>
-        </is>
-      </c>
-    </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Your water quality</t>
+          <t>Your Water Utility's Annual Report</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>La calidad de su agua</t>
+          <t>Informe Anual de Su Proveedor de Agua</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Your water utility's annual report</t>
+          <t>Your filtered drinking water</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Informe de su empresa suministradora de agua</t>
+          <t>Su agua potable filtrada</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>are based on additional samples from inside your home to compare the water from your indoor tap to the water provided by the water utility.</t>
+          <t>Your filtered drinking water (NTU)</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>se basan en muestras adicionales del interior de su hogar para comparar el agua de su grifo interior con el agua proporcionada por la empresa de agua.</t>
+          <t>Su agua potable filtrada (NTU)</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>are based on all samples taken by WCWH from the community, including more than 100 samples from a total of 33 homes from Bastrop County, Hays County, and Travis County.</t>
+          <t>Your filtered drinking water (mg/L)</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>se basan en todas las muestras tomadas por NCNS de la comunidad, incluidas más de 100 muestras de un total de 33 hogares del condado de Bastrop, el condado de Hays y el condado de Travis.</t>
+          <t>Su agua potable filtrada (mg/L)</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>are based on all samples taken by WCWH from the community, including more than 230 samples from a total of 55 homes from Bastrop County, Hays County, and Travis County.</t>
+          <t>Your filtered drinking water (μg/L)</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>se basan en todas las muestras tomadas por NCNS de la comunidad, incluyendo más de 230 muestras de un total de 55 hogares en los condados de Bastrop, Hays y Travis.</t>
+          <t>Su agua potable filtrada (μg/L)</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>are based on the samples that were collected outside your home and reflect the quality of the water that the water utility company provides to your home at the time the sample was taken.</t>
+          <t>Your kitchen tap</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>se basan en las muestras que se recolectaron fuera de su hogar y reflejan la calidad del agua que la compañía de servicios de agua proporciona a su hogar en el momento en que se tomó la muestra.</t>
+          <t>Su grifo de cocina</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>is based on regulations from the Environmental Protection Agency (EPA) and the Texas Commission on Environmental Quality (TCEQ)</t>
+          <t>Your kitchen tap (NTU)</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>se basa en las regulaciones de la Agencia de Protección Ambiental (EPA) y la Comisión de Calidad Ambiental de Texas (TCEQ).</t>
+          <t>Su grifo de cocina (ntu)</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>mg: milligram</t>
+          <t>Your kitchen tap (mg/L)</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>mg: miligramo</t>
+          <t>Su grifo de cocina (mg/L)</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>Your kitchen tap (μg/L)</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>Su grifo de cocina (μg/L)</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>pH is a scale from 0 to 14 that shows how acidic or basic your water is. Water with a pH below 6.5 is acidic. In Travis County, the water is usually more basic.</t>
+          <t>Your level</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>El pH es una escala de 0 a 14 que muestra qué tan ácida o básica es el agua. El agua con un pH por debajo de 6.5 es ácida. En el condado de Travis, el agua suele ser más básica.</t>
+          <t>Su nivel</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>refers to whether the parameters meet the standards of the Texas Commission on Environmental Quality.</t>
+          <t>Your level (NTU)</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>se refiere a si los parámetros cumplen con los estándares de la Comisión de Calidad Ambiental de Texas.</t>
+          <t>Su nivel (NTU)</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>refers to whether the parameters meet the standards(?) of the Texas Commission on Environmental Quality.</t>
+          <t>Your level (mg/L)</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>se refiere a si las medidas cumplen con la Comisión de Calidad Ambiental de Texas.</t>
+          <t>Su nivel (mg/L)</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>wcwhcommunity@austin.utexas.edu</t>
+          <t>Your level (μg/L)</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>wcwhcommunity@austin.utexas.edu</t>
+          <t>Su nivel (μg/L)</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>Your water quality</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>La calidad de su agua</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
+          <t>Your water utility's annual report</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Informe de su empresa suministradora de agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>are based on additional samples from inside your home to compare the water from your indoor tap to the water provided by the water utility.</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>se basan en muestras adicionales del interior de su hogar para comparar el agua de su grifo interior con el agua proporcionada por la empresa de agua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>are based on all samples taken by WCWH from the community, including more than 100 samples from a total of 33 homes from Bastrop County, Hays County, and Travis County.</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>se basan en todas las muestras tomadas por NCNS de la comunidad, incluidas más de 100 muestras de un total de 33 hogares del condado de Bastrop, el condado de Hays y el condado de Travis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>are based on all samples taken by WCWH from the community, including more than 230 samples from a total of 55 homes from Bastrop County, Hays County, and Travis County.</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>se basan en todas las muestras tomadas por NCNS de la comunidad, incluyendo más de 230 muestras de un total de 55 hogares en los condados de Bastrop, Hays y Travis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>are based on the samples that were collected outside your home and reflect the quality of the water that the water utility company provides to your home at the time the sample was taken.</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>se basan en las muestras que se recolectaron fuera de su hogar y reflejan la calidad del agua que la compañía de servicios de agua proporciona a su hogar en el momento en que se tomó la muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>is based on regulations from the Environmental Protection Agency (EPA) and the Texas Commission on Environmental Quality (TCEQ)</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>se basa en las regulaciones de la Agencia de Protección Ambiental (EPA) y la Comisión de Calidad Ambiental de Texas (TCEQ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>mg: milligram</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>mg: miligramo</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>pH is a scale from 0 to 14 that shows how acidic or basic your water is. Water with a pH below 6.5 is acidic. In Travis County, the water is usually more basic.</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>El pH es una escala de 0 a 14 que muestra qué tan ácida o básica es el agua. El agua con un pH por debajo de 6.5 es ácida. En el condado de Travis, el agua suele ser más básica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>refers to whether the parameters meet the standards of the Texas Commission on Environmental Quality.</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>se refiere a si los parámetros cumplen con los estándares de la Comisión de Calidad Ambiental de Texas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>refers to whether the parameters meet the standards(?) of the Texas Commission on Environmental Quality.</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>se refiere a si las medidas cumplen con la Comisión de Calidad Ambiental de Texas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>wcwhcommunity@austin.utexas.edu</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>wcwhcommunity@austin.utexas.edu</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
           <t>µg: microgram</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr">
+      <c r="B277" t="inlineStr">
         <is>
           <t>µg:microgramo</t>
         </is>

</xml_diff>